<commit_message>
Add map QA stories to feature tracker
</commit_message>
<xml_diff>
--- a/outputs/019eee7f-e0ca-7983-a052-837546af2e02/ourtrips-feature-user-story-tracker.xlsx
+++ b/outputs/019eee7f-e0ca-7983-a052-837546af2e02/ourtrips-feature-user-story-tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0b0fcecd4b5f4f12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="R9d81ac115de845c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="3" r:id="R14e72881f0fa4f3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routes and APIs" sheetId="4" r:id="R28cdbc1199a14ad1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R00066570a0184bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="Ra8db854e968a4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="3" r:id="Re6df43061d7540f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routes and APIs" sheetId="4" r:id="Rd6b8b8e5436b45ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UserStories" displayName="UserStories" ref="A1:M87" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UserStories" displayName="UserStories" ref="A1:M90" headerRowCount="1">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -452,7 +452,7 @@
         <x:v>Stories mapped</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>86</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
         <x:v>Feature inventory</x:v>
@@ -481,7 +481,7 @@
         <x:v>Test every user story</x:v>
       </x:c>
       <x:c r="E6" s="13" t="str">
-        <x:v>Completed</x:v>
+        <x:v>Needs Map Retest</x:v>
       </x:c>
       <x:c r="F6" s="13" t="str">
         <x:v>Codex</x:v>
@@ -490,7 +490,7 @@
         <x:v>Browser/API/test commands</x:v>
       </x:c>
       <x:c r="H6" s="13" t="str">
-        <x:v>All mapped stories now have Pass or documented Blocked status.</x:v>
+        <x:v>Map-click, geocoding, and link-correctness stories added as Needs Retest.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -521,13 +521,13 @@
         <x:v>P1 stories</x:v>
       </x:c>
       <x:c r="B8" s="9" t="n">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D8" s="13" t="str">
         <x:v>Retest every behavior</x:v>
       </x:c>
       <x:c r="E8" s="13" t="str">
-        <x:v>Completed</x:v>
+        <x:v>Needs Map Retest</x:v>
       </x:c>
       <x:c r="F8" s="13" t="str">
         <x:v>Codex</x:v>
@@ -536,7 +536,7 @@
         <x:v>Retest Status and notes</x:v>
       </x:c>
       <x:c r="H8" s="13" t="str">
-        <x:v>Post-fix verify, smoke, API, and targeted interaction checks passed; auth-only branches documented blocked.</x:v>
+        <x:v>Prior post-fix verify, smoke, API, and interaction checks passed; new map-specific cases now queued.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -583,7 +583,7 @@
         <x:v>Last updated</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>Updated 2026-06-22 09:43:10 UTC</x:v>
+        <x:v>Updated 2026-06-22 20:30:38 UTC</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4141,61 +4141,178 @@
       </x:c>
     </x:row>
     <x:row r="87" ht="57" hidden="0" customHeight="1">
-      <x:c r="A87" s="21" t="str">
+      <x:c r="A87" s="20" t="str">
         <x:v>US-086</x:v>
       </x:c>
-      <x:c r="B87" s="21" t="str">
+      <x:c r="B87" s="20" t="str">
         <x:v>Agent Knowledge</x:v>
       </x:c>
-      <x:c r="C87" s="21" t="str">
+      <x:c r="C87" s="20" t="str">
         <x:v>knowledge/</x:v>
       </x:c>
-      <x:c r="D87" s="21" t="str">
+      <x:c r="D87" s="20" t="str">
         <x:v>OKF knowledge bundle</x:v>
       </x:c>
-      <x:c r="E87" s="21" t="str">
+      <x:c r="E87" s="20" t="str">
         <x:v>As the trip-chat agent, I want routed knowledge files to be parseable and canonical.</x:v>
       </x:c>
-      <x:c r="F87" s="21" t="str">
+      <x:c r="F87" s="20" t="str">
         <x:v>Every loaded knowledge markdown concept includes required OKF frontmatter, reserved index/log files stay out of the concept map, local duplicate-copy artifacts are ignored, and routed restaurant/accommodation knowledge formats into the prompt checklist.</x:v>
       </x:c>
-      <x:c r="G87" s="21" t="str">
+      <x:c r="G87" s="20" t="str">
         <x:v>knowledge/*.md; src/lib/agent-knowledge.ts; src/lib/agent-knowledge.test.ts</x:v>
       </x:c>
-      <x:c r="H87" s="21" t="str">
+      <x:c r="H87" s="20" t="str">
         <x:v>Retested</x:v>
       </x:c>
-      <x:c r="I87" s="21" t="str">
+      <x:c r="I87" s="20" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="J87" s="21" t="str">
+      <x:c r="J87" s="20" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="K87" s="21" t="str">
+      <x:c r="K87" s="20" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L87" s="21" t="str">
-        <x:v>2026-06-22</x:v>
-      </x:c>
-      <x:c r="M87" s="21" t="str">
+      <x:c r="L87" s="20" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="M87" s="20" t="str">
         <x:v>Knowledge bundle validation and duplicate-artifact regression test passed; full npm run test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="57" hidden="0" customHeight="1">
+      <x:c r="A88" s="20" t="str">
+        <x:v>US-087</x:v>
+      </x:c>
+      <x:c r="B88" s="20" t="str">
+        <x:v>Maps</x:v>
+      </x:c>
+      <x:c r="C88" s="20" t="str">
+        <x:v>Overview/day maps</x:v>
+      </x:c>
+      <x:c r="D88" s="20" t="str">
+        <x:v>Clickable map markers</x:v>
+      </x:c>
+      <x:c r="E88" s="20" t="str">
+        <x:v>As a traveler, I want map pins, route points, and itinerary place labels to be clickable so I can inspect the matching stop or place.</x:v>
+      </x:c>
+      <x:c r="F88" s="20" t="str">
+        <x:v>Overview and day maps expose interactive markers or equivalent controls; clicking a marker or linked itinerary place focuses the correct map target, opens readable place/stop information, and view-all returns the map to all visible locations.</x:v>
+      </x:c>
+      <x:c r="G88" s="20" t="str">
+        <x:v>src/components/preview/ItineraryMap.tsx; src/components/preview/TripPreview.tsx; src/lib/day-map.ts</x:v>
+      </x:c>
+      <x:c r="H88" s="20" t="str">
+        <x:v>Mapped</x:v>
+      </x:c>
+      <x:c r="I88" s="20" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J88" s="20" t="str">
+        <x:v>Browser/Maps</x:v>
+      </x:c>
+      <x:c r="K88" s="20" t="str">
+        <x:v>Needs Retest</x:v>
+      </x:c>
+      <x:c r="L88" s="20" t="str"/>
+      <x:c r="M88" s="20" t="str">
+        <x:v>Added after map audit prompt. Existing smoke verifies map rendering, but marker click/focus behavior needs a dedicated interaction test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="57" hidden="0" customHeight="1">
+      <x:c r="A89" s="20" t="str">
+        <x:v>US-088</x:v>
+      </x:c>
+      <x:c r="B89" s="20" t="str">
+        <x:v>Maps</x:v>
+      </x:c>
+      <x:c r="C89" s="20" t="str">
+        <x:v>Geocoding/search</x:v>
+      </x:c>
+      <x:c r="D89" s="20" t="str">
+        <x:v>Location accuracy and disambiguation</x:v>
+      </x:c>
+      <x:c r="E89" s="20" t="str">
+        <x:v>As a traveler, I want every hotel, restaurant, activity, and route stop to appear in the correct city/country on the map.</x:v>
+      </x:c>
+      <x:c r="F89" s="20" t="str">
+        <x:v>Stored lat/lng and route atlas coordinates are preferred; search queries include trip/day/city context; location bias/restriction prevents ambiguous names from resolving to unrelated cities; a place like Hotel Casablanca must not resolve to Amsterdam when the itinerary context is Casablanca.</x:v>
+      </x:c>
+      <x:c r="G89" s="20" t="str">
+        <x:v>src/components/preview/ItineraryMap.tsx; src/lib/day-map.ts; src/lib/trip-route.ts; src/lib/day-map.test.ts; src/lib/trip-route.test.ts</x:v>
+      </x:c>
+      <x:c r="H89" s="20" t="str">
+        <x:v>Mapped</x:v>
+      </x:c>
+      <x:c r="I89" s="20" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J89" s="20" t="str">
+        <x:v>Browser/Data</x:v>
+      </x:c>
+      <x:c r="K89" s="20" t="str">
+        <x:v>Needs Retest</x:v>
+      </x:c>
+      <x:c r="L89" s="20" t="str"/>
+      <x:c r="M89" s="20" t="str">
+        <x:v>Existing unit tests cover partial disambiguation, fallback points, known aliases, and context-rich search targets; add explicit ambiguous-hotel fixtures and browser map validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="57" hidden="0" customHeight="1">
+      <x:c r="A90" s="21" t="str">
+        <x:v>US-089</x:v>
+      </x:c>
+      <x:c r="B90" s="21" t="str">
+        <x:v>Maps</x:v>
+      </x:c>
+      <x:c r="C90" s="21" t="str">
+        <x:v>Map details and external links</x:v>
+      </x:c>
+      <x:c r="D90" s="21" t="str">
+        <x:v>Place metadata and map links</x:v>
+      </x:c>
+      <x:c r="E90" s="21" t="str">
+        <x:v>As a traveler, I want map detail cards and external map links to describe the same real-world place shown in the itinerary.</x:v>
+      </x:c>
+      <x:c r="F90" s="21" t="str">
+        <x:v>Map details preserve the intended title, type, day/time context, address when known, place_id/google_maps_url when supplied, and safe external map/search links; links must not use stale coordinates, stale labels, or a nearby-but-wrong result.</x:v>
+      </x:c>
+      <x:c r="G90" s="21" t="str">
+        <x:v>src/components/preview/ItineraryMap.tsx; src/components/preview/TripPreview.tsx; src/lib/types.ts; src/lib/day-map.ts</x:v>
+      </x:c>
+      <x:c r="H90" s="21" t="str">
+        <x:v>Mapped</x:v>
+      </x:c>
+      <x:c r="I90" s="21" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J90" s="21" t="str">
+        <x:v>Browser/Maps</x:v>
+      </x:c>
+      <x:c r="K90" s="21" t="str">
+        <x:v>Needs Retest</x:v>
+      </x:c>
+      <x:c r="L90" s="21" t="str"/>
+      <x:c r="M90" s="21" t="str">
+        <x:v>Added as explicit map QA coverage for correct marker metadata and outbound map links.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="H2:H87">
+    <x:dataValidation type="list" sqref="H2:H90">
       <x:formula1>"Mapped,Testing,Issue Found,Fixed,Retested,Blocked,Done"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I2:I87">
+    <x:dataValidation type="list" sqref="I2:I90">
       <x:formula1>"P1,P2,P3"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K2:K87">
+    <x:dataValidation type="list" sqref="K2:K90">
       <x:formula1>"Not Started,Pass,Fail,Blocked,Needs Retest"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8a1cc15957c4b61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92cd72b9f2624157"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4577,7 +4694,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re30f0f87dd394b5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08655f19fe4a4ebd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5397,7 +5514,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ec0872b6fcd40f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6478dc868da44b64"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>